<commit_message>
feat(dcf-grader): refresh WACC and comps with market data
Real comp metrics (Yahoo / stockanalysis, June 2026) and KPMG ANZ MRP:

- rf 4.25% → 4.90% (AU 10Y, late May 2026)
- ERP 6.00% → 5.50% (KPMG, preferred over Damodaran's 4.23% implied)
- Comp lev β refreshed: EDV 0.41, CCEP 0.35 (CCEP D/E and EV/EBITDA
  partly estimated), CPG 0.64, ARMK 1.20, ALL 0.42 → avg unlevered β
  collapses from 0.72 placeholder to 0.30 (peers are much less risky
  than my initial guess)
- Exit multiple: median EV/EBITDA 10.5x → 12.96x

WACC falls 10.05% → 8.07%, EV rises:
- Perpetuity:    $776m → $1,053m
- Exit-multiple: $1,317m → $1,728m

Synced template (Assumptions tab comp values), model-answer doc, and
the grader's MODEL_ANSWER constant. Still staged on branch — not
deployed.

https://claude.ai/code/session_01TeMvKKt5tH7k4HWonJYBxm
</commit_message>
<xml_diff>
--- a/dcf-grader/sample-models/tap-turf-completed-clean.xlsx
+++ b/dcf-grader/sample-models/tap-turf-completed-clean.xlsx
@@ -705,10 +705,10 @@
         </is>
       </c>
       <c r="C20" s="8" t="n">
-        <v>0.85</v>
+        <v>0.41</v>
       </c>
       <c r="D20" s="9" t="n">
-        <v>0.35</v>
+        <v>1.34</v>
       </c>
       <c r="E20" s="10">
         <f>C20/(1+(1-$C$14)*D20)</f>
@@ -722,10 +722,10 @@
         </is>
       </c>
       <c r="C21" s="8" t="n">
-        <v>0.9</v>
+        <v>0.35</v>
       </c>
       <c r="D21" s="9" t="n">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
       <c r="E21" s="10">
         <f>C21/(1+(1-$C$14)*D21)</f>
@@ -739,10 +739,10 @@
         </is>
       </c>
       <c r="C22" s="8" t="n">
-        <v>0.95</v>
+        <v>0.64</v>
       </c>
       <c r="D22" s="9" t="n">
-        <v>0.3</v>
+        <v>1.13</v>
       </c>
       <c r="E22" s="10">
         <f>C22/(1+(1-$C$14)*D22)</f>
@@ -756,10 +756,10 @@
         </is>
       </c>
       <c r="C23" s="8" t="n">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
       <c r="D23" s="9" t="n">
-        <v>0.8</v>
+        <v>2.14</v>
       </c>
       <c r="E23" s="10">
         <f>C23/(1+(1-$C$14)*D23)</f>
@@ -773,10 +773,10 @@
         </is>
       </c>
       <c r="C24" s="8" t="n">
-        <v>0.95</v>
+        <v>0.42</v>
       </c>
       <c r="D24" s="9" t="n">
-        <v>0.15</v>
+        <v>0.31</v>
       </c>
       <c r="E24" s="10">
         <f>C24/(1+(1-$C$14)*D24)</f>
@@ -801,7 +801,7 @@
         </is>
       </c>
       <c r="C27" s="5" t="n">
-        <v>0.0425</v>
+        <v>0.049</v>
       </c>
     </row>
     <row r="28">
@@ -811,7 +811,7 @@
         </is>
       </c>
       <c r="C28" s="5" t="n">
-        <v>0.06</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="29">

</xml_diff>

<commit_message>
data(dcf-grader): replace CCEP estimates with real values
Found CCEP's real metrics: β 0.38, D/E 1.41, EV/EBITDA 13.28×
(stockanalysis.com). All five comps now from real public data, no
estimates remaining.

Impact (minor):
- Avg unlev β: 0.304 → 0.297 → WACC 8.07% → 8.03%
- Median EV/EBITDA: 12.96× → 13.28×
- EV perpetuity:    $1,053m → $1,060m
- EV exit-multiple: $1,728m → $1,768m

Synced: tap-turf-dcf.py, template xlsx, clean xlsx,
tap-turf-model-answer.md, grade-dcf/index.ts MODEL_ANSWER.

https://claude.ai/code/session_01TeMvKKt5tH7k4HWonJYBxm
</commit_message>
<xml_diff>
--- a/dcf-grader/sample-models/tap-turf-completed-clean.xlsx
+++ b/dcf-grader/sample-models/tap-turf-completed-clean.xlsx
@@ -722,10 +722,10 @@
         </is>
       </c>
       <c r="C21" s="8" t="n">
-        <v>0.35</v>
+        <v>0.38</v>
       </c>
       <c r="D21" s="9" t="n">
-        <v>0.8</v>
+        <v>1.41</v>
       </c>
       <c r="E21" s="10">
         <f>C21/(1+(1-$C$14)*D21)</f>

</xml_diff>